<commit_message>
Rename Taxa to Tai and clarify contractual vs market rate
Column 4 renamed from Taxa to Tai. Leave blank to use Tai from
Identificacao sheet. Ajuda explains distinction.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sistema/dist/CADASTRO_ATIVO.xlsx
+++ b/sistema/dist/CADASTRO_ATIVO.xlsx
@@ -93,7 +93,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +118,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4A4A4A"/>
       </patternFill>
     </fill>
     <fill>
@@ -152,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -184,16 +189,20 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -703,13 +712,13 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Taxa de Emissao *</t>
+          <t>Tai — Taxa de Emissao *</t>
         </is>
       </c>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>← Taxa contratual em % a.a. (ex: 6.5 para IPCA+6,5%)</t>
+          <t>← Taxa CONTRATUAL em % a.a. (ex: 6.5 p/ IPCA+6,5% | 12.0 p/ PRE 12%)</t>
         </is>
       </c>
     </row>
@@ -772,13 +781,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -788,10 +798,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Data: DD/MM/AAAA   |   Paga Juros: S ou N   |   % Amortizacao: 0 a 100 (coluna inteira deve somar 100 se amortizante, ou 0 se bullet)   |   Taxa: % a.a. contratual (deixe em branco p/ usar a da aba Identificacao)</t>
+          <t>Data: DD/MM/AAAA   |   Paga Juros: S ou N   |   % Amortizacao: soma deve ser 100 (amortizante) ou deixe 0 em tudo e 100 no vencimento (bullet)   |   Tai: taxa CONTRATUAL do ativo em % a.a. — deixe em BRANCO se for igual em todos os periodos (usa o valor da aba Identificacao)</t>
         </is>
       </c>
     </row>
@@ -811,158 +821,157 @@
           <t>% Amortizacao</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Taxa (% a.a.)</t>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Tai — Taxa Contratual (% a.a.)</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>← DEIXAR EM BRANCO na maioria dos casos</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>15/01/2027</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="14" t="n">
-        <v>6.5</v>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>← Em branco = usa Tai da aba Identificacao</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>15/07/2027</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="14" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="D5" s="16" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>15/01/2028</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="14" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="D6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>15/07/2028</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="D7" s="14" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="D7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>15/01/2029</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="D8" s="14" t="n">
-        <v>6.5</v>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>← Preencha so em bonds com step-up (taxa muda por periodo)</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>15/07/2029</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="D9" s="14" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="D9" s="16" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>15/01/2030</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="D10" s="14" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="D10" s="16" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>15/07/2030</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="D11" s="14" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="D11" s="16" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>^ EXEMPLOS — apague essas linhas e cole os dados reais a partir da linha 4 ^</t>
         </is>
@@ -970,9 +979,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B4:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -989,283 +998,342 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>COMO USAR O CADASTRO_ATIVO.xlsx</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr"/>
+      <c r="A2" s="19" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>PASSO 1 — Aba 'Identificacao'</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Preencha os campos amarelos. Os campos com * sao obrigatorios.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Indexador: use exatamente IPCA+ | PRE | CDI+ | %CDI</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Taxa de Emissao: a taxa CONTRATUAL do ativo (ex: 6.5 para IPCA+6,5% a.a.)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  VNE: valor nominal de emissao — quase sempre R$ 1.000,00</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr"/>
+      <c r="A8" s="19" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>PASSO 2 — Aba 'Fluxo_de_Caixa'</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Apague as linhas de exemplo (linhas 4 a 11).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cole a tabela de pagamentos a partir da linha 4.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Voce pode copiar do Bloomberg, de uma planilha propria ou do prospecto.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr"/>
+      <c r="A13" s="19" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  COLUNAS:</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    Data           : data de cada pagamento no formato DD/MM/AAAA</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    Paga Juros     : S se paga cupom nessa data, N se so amortiza</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    % Amortizacao  : quanto do principal e pago (0 a 100).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">                     Bullet: todos 0 exceto o vencimento que tem 100.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">                     Amortizante: ex 25, 25, 25, 25 (soma = 100).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Taxa (% a.a.)  : taxa do periodo (opcional — deixe em branco p/ usar a da aba anterior)</t>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tai (% a.a.)   : Taxa CONTRATUAL do ativo — define o tamanho do cupom.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr"/>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                     Para IPCA+6,5%: coloque 6.5.  Para PRE 12%: coloque 12.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                     DEIXE EM BRANCO na maioria dos casos: o script usa o valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                     de 'Taxa de Emissao' preenchido na aba Identificacao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                     Preencha so em bonds com step-up (taxa muda por periodo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  IMPORTANTE — TAI x TAXA DE MERCADO:</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tai    = taxa CONTRATUAL (define o fluxo de caixa — vai para o CSV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Taxa de mercado = usada depois no Excel: =RF_PU(ticker; TAXA_MERCADO; data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sao coisas diferentes! O Tai e fixo no prospecto; a de mercado oscila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  EXEMPLOS:</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Bullet IPCA+6,5%:      Data      | S | 0  | (branco)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">                          Data      | S | 0  | (branco)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">                          Vencimento| S | 100| (branco)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Amortizante PRE 12%:   Data      | S | 25 | 12.0</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">                          Data      | S | 25 | 12.0</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">                          Data      | S | 25 | 12.0</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">                          Vencimento| S | 25 | 12.0</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="17" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>PASSO 3 — Importar</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Com o arquivo salvo, abra o terminal na pasta 'sistema' e rode:</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    python scripts/importar_planilha.py CADASTRO_ATIVO.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="17" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  O script cria automaticamente o arquivo CSV em fluxos_manual/</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  e o ativo fica disponivel nas funcoes RF_* sem precisar reabrir o Excel.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="17" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="18" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
         <is>
           <t>DICAS</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  - O ticker deve ser unico (ex: nao use o mesmo ticker de um ativo da B3).</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Para CDI+ e %CDI, use a importacao automatica da B3 (importar_fluxos.py).</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    O cadastro manual de CDI nao e suportado pois depende da curva diaria.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Se errar, basta salvar o Excel corrigido e rodar o importar_planilha.py de novo.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Para atualizar o VNA (IPCA): rode rotina_diaria.py no dia a dia.</t>
         </is>

</xml_diff>